<commit_message>
DDT excel Commit 7
</commit_message>
<xml_diff>
--- a/target/test-classes/TestDataFolder/DemoWebShopExcelSheet.xlsx
+++ b/target/test-classes/TestDataFolder/DemoWebShopExcelSheet.xlsx
@@ -13,7 +13,6 @@
   </bookViews>
   <sheets>
     <sheet name="LogInSheet" sheetId="1" r:id="rId1"/>
-    <sheet name="LogInCustomSheet" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>UserName</t>
   </si>
@@ -36,34 +35,19 @@
     <t>Password@1234</t>
   </si>
   <si>
-    <t>themail1@gmail.com</t>
-  </si>
-  <si>
-    <t>themail2@gmail.com</t>
-  </si>
-  <si>
-    <t>themail3@gmail.com</t>
-  </si>
-  <si>
-    <t>themail4@gmail.com</t>
-  </si>
-  <si>
-    <t>themail5@gmail.com</t>
-  </si>
-  <si>
-    <t>themail6@gmail.com</t>
-  </si>
-  <si>
-    <t>themail7@gmail.com</t>
-  </si>
-  <si>
-    <t>themail8@gmail.com</t>
-  </si>
-  <si>
-    <t>themail9@gmail.com</t>
-  </si>
-  <si>
-    <t>themail10@gmail.com</t>
+    <t>1themail@gmail.com</t>
+  </si>
+  <si>
+    <t>2themail@gmail.com</t>
+  </si>
+  <si>
+    <t>3themail@gmail.com</t>
+  </si>
+  <si>
+    <t>4themail@gmail.com</t>
+  </si>
+  <si>
+    <t>5themail@gmail.com</t>
   </si>
   <si>
     <t>Password@1235</t>
@@ -78,19 +62,13 @@
     <t>Password@1238</t>
   </si>
   <si>
-    <t>Password@1239</t>
-  </si>
-  <si>
-    <t>Password@1240</t>
-  </si>
-  <si>
-    <t>Password@1241</t>
-  </si>
-  <si>
-    <t>Password@1242</t>
-  </si>
-  <si>
-    <t>Password@1243</t>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>dummyMail@gmail.com</t>
+  </si>
+  <si>
+    <t>Password@12345</t>
   </si>
 </sst>
 </file>
@@ -434,22 +412,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -457,76 +438,44 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>21</v>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -537,130 +486,9 @@
     <hyperlink ref="A4" r:id="rId4"/>
     <hyperlink ref="A5" r:id="rId5"/>
     <hyperlink ref="A6" r:id="rId6"/>
-    <hyperlink ref="A7" r:id="rId7"/>
-    <hyperlink ref="A8" r:id="rId8"/>
-    <hyperlink ref="A9" r:id="rId9"/>
-    <hyperlink ref="A10" r:id="rId10"/>
-    <hyperlink ref="A11" r:id="rId11"/>
-    <hyperlink ref="B3:B11" r:id="rId12" display="Password@1234"/>
+    <hyperlink ref="B3:B6" r:id="rId7" display="Password@1234"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId13"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="G5:H15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="7" max="7" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="5" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G15" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="H6" r:id="rId1"/>
-    <hyperlink ref="G6" r:id="rId2"/>
-    <hyperlink ref="G7" r:id="rId3"/>
-    <hyperlink ref="G8" r:id="rId4"/>
-    <hyperlink ref="G9" r:id="rId5"/>
-    <hyperlink ref="G10" r:id="rId6"/>
-    <hyperlink ref="G11" r:id="rId7"/>
-    <hyperlink ref="G12" r:id="rId8"/>
-    <hyperlink ref="G13" r:id="rId9"/>
-    <hyperlink ref="G14" r:id="rId10"/>
-    <hyperlink ref="G15" r:id="rId11"/>
-    <hyperlink ref="H7:H15" r:id="rId12" display="Password@1234"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>